<commit_message>
updated io and analysis outputs from old versions
</commit_message>
<xml_diff>
--- a/LAFExamples/analysis/3-2-scores-trust.xlsx
+++ b/LAFExamples/analysis/3-2-scores-trust.xlsx
@@ -26,79 +26,79 @@
     <t>#Arg-</t>
   </si>
   <si>
-    <t>L17: log4j versions2.0-beta through 2.17.0 are vulnerable</t>
-  </si>
-  <si>
-    <t>L2: security fixes are 2.3.2 and 2.12.4</t>
-  </si>
-  <si>
-    <t>L7: dependencies not in *.java</t>
-  </si>
-  <si>
-    <t>L8: log4j version2.0...2.17.0</t>
-  </si>
-  <si>
-    <t>L11: Steps how to search  on GitHub as user</t>
-  </si>
-  <si>
-    <t>L19: 7 URLs of unknown repositories</t>
-  </si>
-  <si>
-    <t>L16: log4j version:2.0..2.17.0 -2.3.2 -2.12.4</t>
-  </si>
-  <si>
-    <t>L13: most empty, none with gradle, none in right version</t>
-  </si>
-  <si>
-    <t>L23: most empty, none with gradle, one in 2.17.0 version</t>
-  </si>
-  <si>
-    <t>L24: 5 URLs of unknown repositories</t>
-  </si>
-  <si>
-    <t>L14: log4j filename:*.java</t>
-  </si>
-  <si>
-    <t>L0: log4j filename:build.gradle</t>
-  </si>
-  <si>
-    <t>L18: log4j filename:pom.xml</t>
-  </si>
-  <si>
-    <t>L12: dependecies are in build files</t>
-  </si>
-  <si>
-    <t>L10: mostly too new log4j version</t>
-  </si>
-  <si>
-    <t>L20: ~2k repositories</t>
-  </si>
-  <si>
-    <t>L6: Short description how to inspect usage of library in one repository</t>
-  </si>
-  <si>
-    <t>L3: GitHub search cannot search for library versions</t>
-  </si>
-  <si>
-    <t>L25: log4j filename:build.gradle "2.0" "2.1" "2.2" "2.3" "2.4" "2.5" "2.6" "2.7" "2.8" "2.9" "2.10""2.11" "2.12" "2.13" "2.14" "2.15" "2.16" "2.17"</t>
-  </si>
-  <si>
-    <t>L9: GitHub search can search for library versions</t>
-  </si>
-  <si>
-    <t>L4: 0 results, wrong query</t>
-  </si>
-  <si>
-    <t>L15: log4j filename:build.gradle 2.0..2.17.0</t>
-  </si>
-  <si>
-    <t>L1: most empty, none with gradle, two in right versions</t>
-  </si>
-  <si>
-    <t>L21: 12 URLs of unknown repositories</t>
-  </si>
-  <si>
-    <t>L22: engage with community</t>
+    <t>L7: log4j versions2.0-beta through 2.17.0 are vulnerable</t>
+  </si>
+  <si>
+    <t>L8: security fixes are 2.3.2 and 2.12.4</t>
+  </si>
+  <si>
+    <t>L11: dependencies not in *.java</t>
+  </si>
+  <si>
+    <t>L18: log4j version2.0...2.17.0</t>
+  </si>
+  <si>
+    <t>L16: Steps how to search  on GitHub as user</t>
+  </si>
+  <si>
+    <t>L13: 7 URLs of unknown repositories</t>
+  </si>
+  <si>
+    <t>L22: log4j version:2.0..2.17.0 -2.3.2 -2.12.4</t>
+  </si>
+  <si>
+    <t>L23: most empty, none with gradle, none in right version</t>
+  </si>
+  <si>
+    <t>L14: most empty, none with gradle, one in 2.17.0 version</t>
+  </si>
+  <si>
+    <t>L0: 5 URLs of unknown repositories</t>
+  </si>
+  <si>
+    <t>L17: log4j filename:*.java</t>
+  </si>
+  <si>
+    <t>L12: log4j filename:build.gradle</t>
+  </si>
+  <si>
+    <t>L10: log4j filename:pom.xml</t>
+  </si>
+  <si>
+    <t>L19: dependecies are in build files</t>
+  </si>
+  <si>
+    <t>L6: mostly too new log4j version</t>
+  </si>
+  <si>
+    <t>L2: ~2k repositories</t>
+  </si>
+  <si>
+    <t>L24: Short description how to inspect usage of library in one repository</t>
+  </si>
+  <si>
+    <t>L9: GitHub search cannot search for library versions</t>
+  </si>
+  <si>
+    <t>L3: log4j filename:build.gradle "2.0" "2.1" "2.2" "2.3" "2.4" "2.5" "2.6" "2.7" "2.8" "2.9" "2.10""2.11" "2.12" "2.13" "2.14" "2.15" "2.16" "2.17"</t>
+  </si>
+  <si>
+    <t>L15: GitHub search can search for library versions</t>
+  </si>
+  <si>
+    <t>L1: 0 results, wrong query</t>
+  </si>
+  <si>
+    <t>L20: log4j filename:build.gradle 2.0..2.17.0</t>
+  </si>
+  <si>
+    <t>L21: most empty, none with gradle, two in right versions</t>
+  </si>
+  <si>
+    <t>L4: 12 URLs of unknown repositories</t>
+  </si>
+  <si>
+    <t>L25: engage with community</t>
   </si>
   <si>
     <t>L5: utilize dependency management tool</t>
@@ -116,13 +116,13 @@
     <t>logAccumulator</t>
   </si>
   <si>
+    <t>[1.0]</t>
+  </si>
+  <si>
     <t>[]</t>
   </si>
   <si>
     <t>[1.0, 1.0]</t>
-  </si>
-  <si>
-    <t>[1.0]</t>
   </si>
   <si>
     <t>[0.5]</t>
@@ -420,7 +420,7 @@
     <col min="5" max="5" width="8.07421875" customWidth="true" bestFit="true"/>
     <col min="8" max="8" width="11.63671875" customWidth="true" bestFit="true"/>
     <col min="1" max="1" width="2.9296875" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="115.19921875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="114.19921875" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="1.9296875" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="1.9296875" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="8.07421875" customWidth="true" bestFit="true"/>
@@ -488,16 +488,16 @@
         <v>0.0</v>
       </c>
       <c r="E3" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G3" t="n" s="5">
         <v>0.6931471824645996</v>
       </c>
       <c r="H3" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I3" t="s" s="0">
         <v>37</v>
@@ -520,16 +520,16 @@
         <v>0.0</v>
       </c>
       <c r="E4" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G4" t="n" s="5">
         <v>0.6931471824645996</v>
       </c>
       <c r="H4" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I4" t="s" s="0">
         <v>37</v>
@@ -552,16 +552,16 @@
         <v>0.0</v>
       </c>
       <c r="E5" t="s" s="15">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G5" t="n" s="5">
         <v>1.0986123085021973</v>
       </c>
       <c r="H5" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I5" t="s" s="0">
         <v>39</v>
@@ -584,10 +584,10 @@
         <v>1.0</v>
       </c>
       <c r="E6" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G6" t="n" s="7">
         <v>0.0</v>
@@ -616,7 +616,7 @@
         <v>1.0</v>
       </c>
       <c r="E7" t="s" s="15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F7" t="s" s="0">
         <v>37</v>
@@ -628,7 +628,7 @@
         <v>37</v>
       </c>
       <c r="I7" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J7" t="n" s="6">
         <v>-0.28768208622932434</v>
@@ -648,16 +648,16 @@
         <v>0.0</v>
       </c>
       <c r="E8" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F8" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G8" t="n" s="5">
         <v>0.6931471824645996</v>
       </c>
       <c r="H8" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I8" t="s" s="0">
         <v>37</v>
@@ -680,10 +680,10 @@
         <v>1.0</v>
       </c>
       <c r="E9" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F9" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G9" t="n" s="7">
         <v>0.0</v>
@@ -712,19 +712,19 @@
         <v>0.0</v>
       </c>
       <c r="E10" t="s" s="15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F10" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G10" t="n" s="7">
         <v>0.0</v>
       </c>
       <c r="H10" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I10" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J10" t="n" s="7">
         <v>0.0</v>
@@ -744,19 +744,19 @@
         <v>0.0</v>
       </c>
       <c r="E11" t="s" s="15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F11" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G11" t="n" s="7">
         <v>0.0</v>
       </c>
       <c r="H11" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I11" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J11" t="n" s="7">
         <v>0.0</v>
@@ -776,16 +776,16 @@
         <v>0.0</v>
       </c>
       <c r="E12" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F12" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G12" t="n" s="5">
         <v>0.6931471824645996</v>
       </c>
       <c r="H12" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I12" t="s" s="0">
         <v>37</v>
@@ -808,10 +808,10 @@
         <v>2.0</v>
       </c>
       <c r="E13" t="s" s="15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F13" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G13" t="n" s="6">
         <v>-1.0986123085021973</v>
@@ -820,7 +820,7 @@
         <v>39</v>
       </c>
       <c r="I13" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J13" t="n" s="6">
         <v>-0.4054650664329529</v>
@@ -840,10 +840,10 @@
         <v>2.0</v>
       </c>
       <c r="E14" t="s" s="15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F14" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G14" t="n" s="6">
         <v>-1.0986123085021973</v>
@@ -852,7 +852,7 @@
         <v>39</v>
       </c>
       <c r="I14" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J14" t="n" s="6">
         <v>-0.4054650664329529</v>
@@ -872,19 +872,19 @@
         <v>0.0</v>
       </c>
       <c r="E15" t="s" s="15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F15" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G15" t="n" s="7">
         <v>0.0</v>
       </c>
       <c r="H15" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I15" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J15" t="n" s="7">
         <v>0.0</v>
@@ -904,19 +904,19 @@
         <v>0.0</v>
       </c>
       <c r="E16" t="s" s="15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F16" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G16" t="n" s="7">
         <v>0.0</v>
       </c>
       <c r="H16" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I16" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J16" t="n" s="7">
         <v>0.0</v>
@@ -936,19 +936,19 @@
         <v>0.0</v>
       </c>
       <c r="E17" t="s" s="15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F17" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G17" t="n" s="7">
         <v>0.0</v>
       </c>
       <c r="H17" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I17" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J17" t="n" s="7">
         <v>0.0</v>
@@ -968,19 +968,19 @@
         <v>0.0</v>
       </c>
       <c r="E18" t="s" s="15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F18" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G18" t="n" s="7">
         <v>0.0</v>
       </c>
       <c r="H18" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I18" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J18" t="n" s="7">
         <v>0.0</v>
@@ -1000,19 +1000,19 @@
         <v>0.0</v>
       </c>
       <c r="E19" t="s" s="15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F19" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G19" t="n" s="7">
         <v>0.0</v>
       </c>
       <c r="H19" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I19" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J19" t="n" s="7">
         <v>0.0</v>
@@ -1032,10 +1032,10 @@
         <v>1.0</v>
       </c>
       <c r="E20" t="s" s="15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F20" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G20" t="n" s="6">
         <v>-0.6931471824645996</v>
@@ -1044,7 +1044,7 @@
         <v>37</v>
       </c>
       <c r="I20" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J20" t="n" s="6">
         <v>-0.28768208622932434</v>
@@ -1064,10 +1064,10 @@
         <v>1.0</v>
       </c>
       <c r="E21" t="s" s="15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F21" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G21" t="n" s="6">
         <v>-0.6931471824645996</v>
@@ -1076,7 +1076,7 @@
         <v>37</v>
       </c>
       <c r="I21" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J21" t="n" s="6">
         <v>-0.28768208622932434</v>
@@ -1096,19 +1096,19 @@
         <v>0.0</v>
       </c>
       <c r="E22" t="s" s="15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F22" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G22" t="n" s="7">
         <v>0.0</v>
       </c>
       <c r="H22" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I22" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J22" t="n" s="7">
         <v>0.0</v>
@@ -1128,19 +1128,19 @@
         <v>0.0</v>
       </c>
       <c r="E23" t="s" s="15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F23" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G23" t="n" s="7">
         <v>0.0</v>
       </c>
       <c r="H23" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I23" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J23" t="n" s="7">
         <v>0.0</v>
@@ -1160,10 +1160,10 @@
         <v>1.0</v>
       </c>
       <c r="E24" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F24" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G24" t="n" s="7">
         <v>0.0</v>
@@ -1192,19 +1192,19 @@
         <v>0.0</v>
       </c>
       <c r="E25" t="s" s="15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F25" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G25" t="n" s="7">
         <v>0.0</v>
       </c>
       <c r="H25" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I25" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J25" t="n" s="7">
         <v>0.0</v>
@@ -1224,19 +1224,19 @@
         <v>0.0</v>
       </c>
       <c r="E26" t="s" s="15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F26" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G26" t="n" s="7">
         <v>0.0</v>
       </c>
       <c r="H26" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I26" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J26" t="n" s="7">
         <v>0.0</v>
@@ -1256,19 +1256,19 @@
         <v>0.0</v>
       </c>
       <c r="E27" t="s" s="15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F27" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G27" t="n" s="7">
         <v>0.0</v>
       </c>
       <c r="H27" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I27" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J27" t="n" s="7">
         <v>0.0</v>
@@ -1288,19 +1288,19 @@
         <v>0.0</v>
       </c>
       <c r="E28" t="s" s="15">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F28" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G28" t="n" s="7">
         <v>0.0</v>
       </c>
       <c r="H28" t="s" s="15">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="I28" t="s" s="0">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="J28" t="n" s="7">
         <v>0.0</v>

</xml_diff>